<commit_message>
fix(security-audit): sanitize compose environment variables, enforce explicit DATABASE_URL checks, update XML formula metric formulation, and align gatekeeper status
</commit_message>
<xml_diff>
--- a/docs/validation/evidence/payroll/reference-provisions-2026.xlsx
+++ b/docs/validation/evidence/payroll/reference-provisions-2026.xlsx
@@ -12531,9 +12531,8 @@
         <f>'Détails'!AI2</f>
         <v>PASS</v>
       </c>
-      <c r="AH2" t="str">
+      <c r="AH2">
         <f>'Détails'!AJ2</f>
-        <v/>
       </c>
     </row>
     <row r="3">
@@ -12667,9 +12666,8 @@
         <f>'Détails'!AI3</f>
         <v>PASS</v>
       </c>
-      <c r="AH3" t="str">
+      <c r="AH3">
         <f>'Détails'!AJ3</f>
-        <v/>
       </c>
     </row>
     <row r="4">
@@ -12803,9 +12801,8 @@
         <f>'Détails'!AI4</f>
         <v>PASS</v>
       </c>
-      <c r="AH4" t="str">
+      <c r="AH4">
         <f>'Détails'!AJ4</f>
-        <v/>
       </c>
     </row>
     <row r="5">
@@ -12939,9 +12936,8 @@
         <f>'Détails'!AI5</f>
         <v>PASS</v>
       </c>
-      <c r="AH5" t="str">
+      <c r="AH5">
         <f>'Détails'!AJ5</f>
-        <v/>
       </c>
     </row>
     <row r="6">
@@ -13075,9 +13071,8 @@
         <f>'Détails'!AI6</f>
         <v>PASS</v>
       </c>
-      <c r="AH6" t="str">
+      <c r="AH6">
         <f>'Détails'!AJ6</f>
-        <v/>
       </c>
     </row>
     <row r="7">
@@ -13211,9 +13206,8 @@
         <f>'Détails'!AI7</f>
         <v>PASS</v>
       </c>
-      <c r="AH7" t="str">
+      <c r="AH7">
         <f>'Détails'!AJ7</f>
-        <v/>
       </c>
     </row>
     <row r="8">
@@ -13347,9 +13341,8 @@
         <f>'Détails'!AI8</f>
         <v>PASS</v>
       </c>
-      <c r="AH8" t="str">
+      <c r="AH8">
         <f>'Détails'!AJ8</f>
-        <v/>
       </c>
     </row>
     <row r="9">
@@ -13483,9 +13476,8 @@
         <f>'Détails'!AI9</f>
         <v>PASS</v>
       </c>
-      <c r="AH9" t="str">
+      <c r="AH9">
         <f>'Détails'!AJ9</f>
-        <v/>
       </c>
     </row>
     <row r="10">
@@ -13619,9 +13611,8 @@
         <f>'Détails'!AI10</f>
         <v>PASS</v>
       </c>
-      <c r="AH10" t="str">
+      <c r="AH10">
         <f>'Détails'!AJ10</f>
-        <v/>
       </c>
     </row>
     <row r="11">
@@ -13755,9 +13746,8 @@
         <f>'Détails'!AI11</f>
         <v>PASS</v>
       </c>
-      <c r="AH11" t="str">
+      <c r="AH11">
         <f>'Détails'!AJ11</f>
-        <v/>
       </c>
     </row>
     <row r="12">
@@ -13891,9 +13881,8 @@
         <f>'Détails'!AI12</f>
         <v>PASS</v>
       </c>
-      <c r="AH12" t="str">
+      <c r="AH12">
         <f>'Détails'!AJ12</f>
-        <v/>
       </c>
     </row>
     <row r="13">
@@ -14027,9 +14016,8 @@
         <f>'Détails'!AI13</f>
         <v>PASS</v>
       </c>
-      <c r="AH13" t="str">
+      <c r="AH13">
         <f>'Détails'!AJ13</f>
-        <v/>
       </c>
     </row>
     <row r="14">
@@ -14435,9 +14423,8 @@
         <f>'Détails'!AI16</f>
         <v>PASS</v>
       </c>
-      <c r="AH16" t="str">
+      <c r="AH16">
         <f>'Détails'!AJ16</f>
-        <v/>
       </c>
     </row>
     <row r="17">
@@ -14571,9 +14558,8 @@
         <f>'Détails'!AI17</f>
         <v>PASS</v>
       </c>
-      <c r="AH17" t="str">
+      <c r="AH17">
         <f>'Détails'!AJ17</f>
-        <v/>
       </c>
     </row>
     <row r="18">
@@ -14707,9 +14693,8 @@
         <f>'Détails'!AI18</f>
         <v>PASS</v>
       </c>
-      <c r="AH18" t="str">
+      <c r="AH18">
         <f>'Détails'!AJ18</f>
-        <v/>
       </c>
     </row>
     <row r="19">
@@ -14979,9 +14964,8 @@
         <f>'Détails'!AI20</f>
         <v>PASS</v>
       </c>
-      <c r="AH20" t="str">
+      <c r="AH20">
         <f>'Détails'!AJ20</f>
-        <v/>
       </c>
     </row>
     <row r="21">
@@ -15115,9 +15099,8 @@
         <f>'Détails'!AI21</f>
         <v>PASS</v>
       </c>
-      <c r="AH21" t="str">
+      <c r="AH21">
         <f>'Détails'!AJ21</f>
-        <v/>
       </c>
     </row>
   </sheetData>

</xml_diff>